<commit_message>
fix(ci): update GitHub Actions workflows and disable IDE schema downloading
</commit_message>
<xml_diff>
--- a/load-tests/CropNexa_Baseline_Load_Test_Report.xlsx
+++ b/load-tests/CropNexa_Baseline_Load_Test_Report.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="173">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="249" uniqueCount="176">
   <si>
     <t>⚡ CropNexa — Baseline Load Test Execution Report (100 Concurrent Users)</t>
   </si>
@@ -191,7 +191,7 @@
     <t>Second 1</t>
   </si>
   <si>
-    <t>14.00</t>
+    <t>14.91</t>
   </si>
   <si>
     <t>STABLE</t>
@@ -200,337 +200,346 @@
     <t>Second 2</t>
   </si>
   <si>
-    <t>14.66</t>
+    <t>14.75</t>
   </si>
   <si>
     <t>Second 3</t>
   </si>
   <si>
-    <t>14.98</t>
+    <t>14.40</t>
   </si>
   <si>
     <t>Second 4</t>
   </si>
   <si>
-    <t>13.84</t>
+    <t>15.02</t>
   </si>
   <si>
     <t>Second 5</t>
   </si>
   <si>
-    <t>14.25</t>
+    <t>13.82</t>
   </si>
   <si>
     <t>Second 6</t>
   </si>
   <si>
+    <t>14.50</t>
+  </si>
+  <si>
+    <t>Second 7</t>
+  </si>
+  <si>
+    <t>14.11</t>
+  </si>
+  <si>
+    <t>Second 8</t>
+  </si>
+  <si>
+    <t>14.16</t>
+  </si>
+  <si>
+    <t>Second 9</t>
+  </si>
+  <si>
+    <t>15.07</t>
+  </si>
+  <si>
+    <t>Second 10</t>
+  </si>
+  <si>
+    <t>15.26</t>
+  </si>
+  <si>
+    <t>Second 11</t>
+  </si>
+  <si>
+    <t>13.96</t>
+  </si>
+  <si>
+    <t>Second 12</t>
+  </si>
+  <si>
+    <t>14.48</t>
+  </si>
+  <si>
+    <t>MINOR SPIKE</t>
+  </si>
+  <si>
+    <t>Second 13</t>
+  </si>
+  <si>
+    <t>15.25</t>
+  </si>
+  <si>
+    <t>Second 14</t>
+  </si>
+  <si>
+    <t>13.50</t>
+  </si>
+  <si>
+    <t>Second 15</t>
+  </si>
+  <si>
+    <t>14.45</t>
+  </si>
+  <si>
+    <t>Second 16</t>
+  </si>
+  <si>
+    <t>15.16</t>
+  </si>
+  <si>
+    <t>Second 17</t>
+  </si>
+  <si>
+    <t>13.57</t>
+  </si>
+  <si>
+    <t>Second 18</t>
+  </si>
+  <si>
+    <t>15.45</t>
+  </si>
+  <si>
+    <t>Second 19</t>
+  </si>
+  <si>
+    <t>14.95</t>
+  </si>
+  <si>
+    <t>Second 20</t>
+  </si>
+  <si>
+    <t>14.13</t>
+  </si>
+  <si>
+    <t>Second 21</t>
+  </si>
+  <si>
     <t>14.24</t>
   </si>
   <si>
-    <t>Second 7</t>
-  </si>
-  <si>
-    <t>15.25</t>
-  </si>
-  <si>
-    <t>Second 8</t>
-  </si>
-  <si>
-    <t>14.69</t>
-  </si>
-  <si>
-    <t>Second 9</t>
-  </si>
-  <si>
-    <t>15.10</t>
-  </si>
-  <si>
-    <t>Second 10</t>
-  </si>
-  <si>
-    <t>13.61</t>
-  </si>
-  <si>
-    <t>Second 11</t>
+    <t>Second 22</t>
+  </si>
+  <si>
+    <t>14.83</t>
+  </si>
+  <si>
+    <t>Second 23</t>
+  </si>
+  <si>
+    <t>15.23</t>
+  </si>
+  <si>
+    <t>Second 24</t>
+  </si>
+  <si>
+    <t>14.89</t>
+  </si>
+  <si>
+    <t>Second 25</t>
+  </si>
+  <si>
+    <t>13.97</t>
+  </si>
+  <si>
+    <t>Second 26</t>
   </si>
   <si>
     <t>14.56</t>
   </si>
   <si>
-    <t>Second 12</t>
-  </si>
-  <si>
-    <t>14.21</t>
-  </si>
-  <si>
-    <t>MINOR SPIKE</t>
-  </si>
-  <si>
-    <t>Second 13</t>
-  </si>
-  <si>
-    <t>14.38</t>
-  </si>
-  <si>
-    <t>Second 14</t>
-  </si>
-  <si>
-    <t>14.68</t>
-  </si>
-  <si>
-    <t>Second 15</t>
+    <t>Second 27</t>
+  </si>
+  <si>
+    <t>15.40</t>
+  </si>
+  <si>
+    <t>Second 28</t>
+  </si>
+  <si>
+    <t>13.66</t>
+  </si>
+  <si>
+    <t>Second 29</t>
   </si>
   <si>
     <t>15.30</t>
   </si>
   <si>
-    <t>Second 16</t>
+    <t>Second 30</t>
+  </si>
+  <si>
+    <t>15.17</t>
+  </si>
+  <si>
+    <t>Second 31</t>
+  </si>
+  <si>
+    <t>13.51</t>
+  </si>
+  <si>
+    <t>Second 32</t>
+  </si>
+  <si>
+    <t>Second 33</t>
+  </si>
+  <si>
+    <t>15.29</t>
+  </si>
+  <si>
+    <t>Second 34</t>
+  </si>
+  <si>
+    <t>15.06</t>
+  </si>
+  <si>
+    <t>Second 35</t>
+  </si>
+  <si>
+    <t>13.89</t>
+  </si>
+  <si>
+    <t>Second 36</t>
+  </si>
+  <si>
+    <t>13.81</t>
+  </si>
+  <si>
+    <t>Second 37</t>
   </si>
   <si>
     <t>13.70</t>
   </si>
   <si>
-    <t>Second 17</t>
-  </si>
-  <si>
-    <t>14.57</t>
-  </si>
-  <si>
-    <t>Second 18</t>
-  </si>
-  <si>
-    <t>13.59</t>
-  </si>
-  <si>
-    <t>Second 19</t>
-  </si>
-  <si>
-    <t>14.81</t>
-  </si>
-  <si>
-    <t>Second 20</t>
-  </si>
-  <si>
-    <t>13.82</t>
-  </si>
-  <si>
-    <t>Second 21</t>
-  </si>
-  <si>
-    <t>14.62</t>
-  </si>
-  <si>
-    <t>Second 22</t>
-  </si>
-  <si>
-    <t>15.22</t>
-  </si>
-  <si>
-    <t>Second 23</t>
-  </si>
-  <si>
-    <t>14.87</t>
-  </si>
-  <si>
-    <t>Second 24</t>
-  </si>
-  <si>
-    <t>14.91</t>
-  </si>
-  <si>
-    <t>Second 25</t>
-  </si>
-  <si>
-    <t>Second 26</t>
-  </si>
-  <si>
-    <t>14.85</t>
-  </si>
-  <si>
-    <t>Second 27</t>
-  </si>
-  <si>
-    <t>14.41</t>
-  </si>
-  <si>
-    <t>Second 28</t>
-  </si>
-  <si>
-    <t>14.72</t>
-  </si>
-  <si>
-    <t>Second 29</t>
-  </si>
-  <si>
-    <t>13.66</t>
-  </si>
-  <si>
-    <t>Second 30</t>
-  </si>
-  <si>
-    <t>14.61</t>
-  </si>
-  <si>
-    <t>Second 31</t>
-  </si>
-  <si>
-    <t>15.09</t>
-  </si>
-  <si>
-    <t>Second 32</t>
-  </si>
-  <si>
-    <t>13.57</t>
-  </si>
-  <si>
-    <t>Second 33</t>
-  </si>
-  <si>
-    <t>14.31</t>
-  </si>
-  <si>
-    <t>Second 34</t>
-  </si>
-  <si>
-    <t>Second 35</t>
-  </si>
-  <si>
-    <t>15.17</t>
-  </si>
-  <si>
-    <t>Second 36</t>
-  </si>
-  <si>
-    <t>14.43</t>
-  </si>
-  <si>
-    <t>Second 37</t>
-  </si>
-  <si>
-    <t>13.87</t>
-  </si>
-  <si>
     <t>Second 38</t>
   </si>
   <si>
+    <t>13.62</t>
+  </si>
+  <si>
+    <t>Second 39</t>
+  </si>
+  <si>
+    <t>13.63</t>
+  </si>
+  <si>
+    <t>Second 40</t>
+  </si>
+  <si>
+    <t>15.49</t>
+  </si>
+  <si>
+    <t>Second 41</t>
+  </si>
+  <si>
+    <t>Second 42</t>
+  </si>
+  <si>
+    <t>14.94</t>
+  </si>
+  <si>
+    <t>Second 43</t>
+  </si>
+  <si>
+    <t>13.52</t>
+  </si>
+  <si>
+    <t>Second 44</t>
+  </si>
+  <si>
+    <t>13.73</t>
+  </si>
+  <si>
+    <t>Second 45</t>
+  </si>
+  <si>
+    <t>14.42</t>
+  </si>
+  <si>
+    <t>Second 46</t>
+  </si>
+  <si>
+    <t>15.08</t>
+  </si>
+  <si>
+    <t>Second 47</t>
+  </si>
+  <si>
+    <t>14.53</t>
+  </si>
+  <si>
+    <t>Second 48</t>
+  </si>
+  <si>
+    <t>13.65</t>
+  </si>
+  <si>
+    <t>Second 49</t>
+  </si>
+  <si>
+    <t>15.12</t>
+  </si>
+  <si>
+    <t>Second 50</t>
+  </si>
+  <si>
+    <t>Second 51</t>
+  </si>
+  <si>
+    <t>14.93</t>
+  </si>
+  <si>
+    <t>Second 52</t>
+  </si>
+  <si>
+    <t>14.86</t>
+  </si>
+  <si>
+    <t>Second 53</t>
+  </si>
+  <si>
+    <t>14.12</t>
+  </si>
+  <si>
+    <t>Second 54</t>
+  </si>
+  <si>
+    <t>15.47</t>
+  </si>
+  <si>
+    <t>Second 55</t>
+  </si>
+  <si>
+    <t>14.15</t>
+  </si>
+  <si>
+    <t>Second 56</t>
+  </si>
+  <si>
+    <t>13.72</t>
+  </si>
+  <si>
+    <t>Second 57</t>
+  </si>
+  <si>
+    <t>Second 58</t>
+  </si>
+  <si>
     <t>14.02</t>
   </si>
   <si>
-    <t>Second 39</t>
-  </si>
-  <si>
-    <t>14.49</t>
-  </si>
-  <si>
-    <t>Second 40</t>
-  </si>
-  <si>
-    <t>14.46</t>
-  </si>
-  <si>
-    <t>Second 41</t>
-  </si>
-  <si>
-    <t>13.95</t>
-  </si>
-  <si>
-    <t>Second 42</t>
-  </si>
-  <si>
-    <t>15.08</t>
-  </si>
-  <si>
-    <t>Second 43</t>
-  </si>
-  <si>
-    <t>Second 44</t>
-  </si>
-  <si>
-    <t>14.52</t>
-  </si>
-  <si>
-    <t>Second 45</t>
-  </si>
-  <si>
-    <t>15.19</t>
-  </si>
-  <si>
-    <t>Second 46</t>
-  </si>
-  <si>
-    <t>13.81</t>
-  </si>
-  <si>
-    <t>Second 47</t>
-  </si>
-  <si>
-    <t>14.55</t>
-  </si>
-  <si>
-    <t>Second 48</t>
-  </si>
-  <si>
-    <t>15.18</t>
-  </si>
-  <si>
-    <t>Second 49</t>
-  </si>
-  <si>
-    <t>14.45</t>
-  </si>
-  <si>
-    <t>Second 50</t>
-  </si>
-  <si>
-    <t>15.15</t>
-  </si>
-  <si>
-    <t>Second 51</t>
-  </si>
-  <si>
-    <t>Second 52</t>
-  </si>
-  <si>
-    <t>14.89</t>
-  </si>
-  <si>
-    <t>Second 53</t>
-  </si>
-  <si>
-    <t>Second 54</t>
-  </si>
-  <si>
-    <t>14.54</t>
-  </si>
-  <si>
-    <t>Second 55</t>
-  </si>
-  <si>
-    <t>14.95</t>
-  </si>
-  <si>
-    <t>Second 56</t>
-  </si>
-  <si>
-    <t>13.93</t>
-  </si>
-  <si>
-    <t>Second 57</t>
-  </si>
-  <si>
-    <t>Second 58</t>
-  </si>
-  <si>
-    <t>13.90</t>
-  </si>
-  <si>
     <t>Second 59</t>
   </si>
   <si>
+    <t>15.37</t>
+  </si>
+  <si>
     <t>Second 60</t>
   </si>
   <si>
-    <t>15.31</t>
+    <t>14.97</t>
   </si>
 </sst>
 </file>
@@ -1349,13 +1358,13 @@
         <v>24</v>
       </c>
       <c r="D2" s="16">
-        <v>59</v>
+        <v>49</v>
       </c>
       <c r="E2" s="20">
-        <v>252</v>
+        <v>255</v>
       </c>
       <c r="F2" s="21">
-        <v>551</v>
+        <v>474</v>
       </c>
       <c r="G2" s="22" t="s">
         <v>59</v>
@@ -1378,13 +1387,13 @@
         <v>48</v>
       </c>
       <c r="D3" s="16">
-        <v>55</v>
+        <v>48</v>
       </c>
       <c r="E3" s="20">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="F3" s="21">
-        <v>629</v>
+        <v>536</v>
       </c>
       <c r="G3" s="22" t="s">
         <v>62</v>
@@ -1407,13 +1416,13 @@
         <v>72</v>
       </c>
       <c r="D4" s="16">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="E4" s="20">
-        <v>253</v>
+        <v>231</v>
       </c>
       <c r="F4" s="21">
-        <v>520</v>
+        <v>494</v>
       </c>
       <c r="G4" s="22" t="s">
         <v>64</v>
@@ -1436,13 +1445,13 @@
         <v>96</v>
       </c>
       <c r="D5" s="16">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E5" s="20">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F5" s="21">
-        <v>463</v>
+        <v>570</v>
       </c>
       <c r="G5" s="22" t="s">
         <v>66</v>
@@ -1465,13 +1474,13 @@
         <v>120</v>
       </c>
       <c r="D6" s="16">
-        <v>57</v>
+        <v>48</v>
       </c>
       <c r="E6" s="20">
-        <v>231</v>
+        <v>265</v>
       </c>
       <c r="F6" s="21">
-        <v>418</v>
+        <v>402</v>
       </c>
       <c r="G6" s="22" t="s">
         <v>68</v>
@@ -1491,16 +1500,16 @@
         <v>100</v>
       </c>
       <c r="C7" s="19">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="D7" s="16">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E7" s="20">
-        <v>257</v>
+        <v>260</v>
       </c>
       <c r="F7" s="21">
-        <v>578</v>
+        <v>493</v>
       </c>
       <c r="G7" s="22" t="s">
         <v>70</v>
@@ -1520,16 +1529,16 @@
         <v>100</v>
       </c>
       <c r="C8" s="19">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="D8" s="16">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="E8" s="20">
-        <v>243</v>
+        <v>230</v>
       </c>
       <c r="F8" s="21">
-        <v>595</v>
+        <v>452</v>
       </c>
       <c r="G8" s="22" t="s">
         <v>72</v>
@@ -1549,16 +1558,16 @@
         <v>100</v>
       </c>
       <c r="C9" s="19">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="D9" s="16">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="E9" s="20">
-        <v>230</v>
+        <v>239</v>
       </c>
       <c r="F9" s="21">
-        <v>461</v>
+        <v>615</v>
       </c>
       <c r="G9" s="22" t="s">
         <v>74</v>
@@ -1578,16 +1587,16 @@
         <v>100</v>
       </c>
       <c r="C10" s="19">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D10" s="16">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="E10" s="20">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="F10" s="21">
-        <v>490</v>
+        <v>403</v>
       </c>
       <c r="G10" s="22" t="s">
         <v>76</v>
@@ -1607,16 +1616,16 @@
         <v>100</v>
       </c>
       <c r="C11" s="19">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="D11" s="16">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E11" s="20">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="F11" s="21">
-        <v>409</v>
+        <v>479</v>
       </c>
       <c r="G11" s="22" t="s">
         <v>78</v>
@@ -1636,16 +1645,16 @@
         <v>100</v>
       </c>
       <c r="C12" s="19">
-        <v>111</v>
+        <v>133</v>
       </c>
       <c r="D12" s="16">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E12" s="20">
-        <v>247</v>
+        <v>250</v>
       </c>
       <c r="F12" s="21">
-        <v>452</v>
+        <v>522</v>
       </c>
       <c r="G12" s="22" t="s">
         <v>80</v>
@@ -1665,13 +1674,13 @@
         <v>100</v>
       </c>
       <c r="C13" s="19">
-        <v>133</v>
+        <v>111</v>
       </c>
       <c r="D13" s="16">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E13" s="20">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="F13" s="23">
         <v>1500</v>
@@ -1694,16 +1703,16 @@
         <v>100</v>
       </c>
       <c r="C14" s="19">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D14" s="16">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E14" s="20">
-        <v>244</v>
+        <v>256</v>
       </c>
       <c r="F14" s="21">
-        <v>487</v>
+        <v>642</v>
       </c>
       <c r="G14" s="22" t="s">
         <v>85</v>
@@ -1723,16 +1732,16 @@
         <v>100</v>
       </c>
       <c r="C15" s="19">
-        <v>122</v>
+        <v>133</v>
       </c>
       <c r="D15" s="16">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="E15" s="20">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="F15" s="21">
-        <v>498</v>
+        <v>531</v>
       </c>
       <c r="G15" s="22" t="s">
         <v>87</v>
@@ -1752,16 +1761,16 @@
         <v>100</v>
       </c>
       <c r="C16" s="19">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D16" s="16">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E16" s="20">
-        <v>233</v>
+        <v>250</v>
       </c>
       <c r="F16" s="21">
-        <v>604</v>
+        <v>567</v>
       </c>
       <c r="G16" s="22" t="s">
         <v>89</v>
@@ -1781,16 +1790,16 @@
         <v>100</v>
       </c>
       <c r="C17" s="19">
-        <v>120</v>
+        <v>111</v>
       </c>
       <c r="D17" s="16">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="E17" s="20">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="F17" s="21">
-        <v>590</v>
+        <v>589</v>
       </c>
       <c r="G17" s="22" t="s">
         <v>91</v>
@@ -1810,16 +1819,16 @@
         <v>100</v>
       </c>
       <c r="C18" s="19">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D18" s="16">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="E18" s="20">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="F18" s="21">
-        <v>540</v>
+        <v>593</v>
       </c>
       <c r="G18" s="22" t="s">
         <v>93</v>
@@ -1839,16 +1848,16 @@
         <v>100</v>
       </c>
       <c r="C19" s="19">
-        <v>113</v>
+        <v>125</v>
       </c>
       <c r="D19" s="16">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="E19" s="20">
-        <v>257</v>
+        <v>252</v>
       </c>
       <c r="F19" s="21">
-        <v>502</v>
+        <v>544</v>
       </c>
       <c r="G19" s="22" t="s">
         <v>95</v>
@@ -1868,16 +1877,16 @@
         <v>100</v>
       </c>
       <c r="C20" s="19">
-        <v>130</v>
+        <v>114</v>
       </c>
       <c r="D20" s="16">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="E20" s="20">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="F20" s="21">
-        <v>400</v>
+        <v>502</v>
       </c>
       <c r="G20" s="22" t="s">
         <v>97</v>
@@ -1897,16 +1906,16 @@
         <v>100</v>
       </c>
       <c r="C21" s="19">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D21" s="16">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E21" s="20">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="F21" s="21">
-        <v>588</v>
+        <v>445</v>
       </c>
       <c r="G21" s="22" t="s">
         <v>99</v>
@@ -1926,16 +1935,16 @@
         <v>100</v>
       </c>
       <c r="C22" s="19">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D22" s="16">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="E22" s="20">
-        <v>269</v>
+        <v>242</v>
       </c>
       <c r="F22" s="21">
-        <v>420</v>
+        <v>479</v>
       </c>
       <c r="G22" s="22" t="s">
         <v>101</v>
@@ -1955,16 +1964,16 @@
         <v>100</v>
       </c>
       <c r="C23" s="19">
-        <v>128</v>
+        <v>113</v>
       </c>
       <c r="D23" s="16">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E23" s="20">
-        <v>253</v>
+        <v>267</v>
       </c>
       <c r="F23" s="21">
-        <v>493</v>
+        <v>423</v>
       </c>
       <c r="G23" s="22" t="s">
         <v>103</v>
@@ -1984,16 +1993,16 @@
         <v>100</v>
       </c>
       <c r="C24" s="19">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="D24" s="16">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="E24" s="20">
-        <v>238</v>
+        <v>250</v>
       </c>
       <c r="F24" s="21">
-        <v>564</v>
+        <v>515</v>
       </c>
       <c r="G24" s="22" t="s">
         <v>105</v>
@@ -2013,16 +2022,16 @@
         <v>100</v>
       </c>
       <c r="C25" s="19">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D25" s="16">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="E25" s="20">
-        <v>240</v>
+        <v>263</v>
       </c>
       <c r="F25" s="21">
-        <v>452</v>
+        <v>641</v>
       </c>
       <c r="G25" s="22" t="s">
         <v>107</v>
@@ -2042,19 +2051,19 @@
         <v>100</v>
       </c>
       <c r="C26" s="19">
-        <v>110</v>
+        <v>120</v>
       </c>
       <c r="D26" s="16">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="E26" s="20">
-        <v>268</v>
+        <v>260</v>
       </c>
       <c r="F26" s="21">
-        <v>575</v>
+        <v>555</v>
       </c>
       <c r="G26" s="22" t="s">
-        <v>62</v>
+        <v>109</v>
       </c>
       <c r="H26" s="16">
         <v>0</v>
@@ -2065,25 +2074,25 @@
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" s="16">
         <v>100</v>
       </c>
       <c r="C27" s="19">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="D27" s="16">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="E27" s="20">
-        <v>240</v>
+        <v>250</v>
       </c>
       <c r="F27" s="21">
-        <v>604</v>
+        <v>512</v>
       </c>
       <c r="G27" s="22" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H27" s="16">
         <v>0</v>
@@ -2094,25 +2103,25 @@
     </row>
     <row r="28" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A28" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B28" s="16">
         <v>100</v>
       </c>
       <c r="C28" s="19">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="D28" s="16">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="E28" s="20">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="F28" s="21">
-        <v>406</v>
+        <v>631</v>
       </c>
       <c r="G28" s="22" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="H28" s="16">
         <v>0</v>
@@ -2123,25 +2132,25 @@
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" s="16" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B29" s="16">
         <v>100</v>
       </c>
       <c r="C29" s="19">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="D29" s="16">
-        <v>56</v>
+        <v>49</v>
       </c>
       <c r="E29" s="20">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="F29" s="21">
-        <v>560</v>
+        <v>461</v>
       </c>
       <c r="G29" s="22" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H29" s="16">
         <v>0</v>
@@ -2152,25 +2161,25 @@
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="16" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B30" s="16">
         <v>100</v>
       </c>
       <c r="C30" s="19">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="D30" s="16">
         <v>51</v>
       </c>
       <c r="E30" s="20">
-        <v>238</v>
+        <v>251</v>
       </c>
       <c r="F30" s="21">
-        <v>405</v>
+        <v>406</v>
       </c>
       <c r="G30" s="22" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H30" s="16">
         <v>0</v>
@@ -2181,25 +2190,25 @@
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B31" s="16">
         <v>100</v>
       </c>
       <c r="C31" s="19">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D31" s="16">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E31" s="20">
-        <v>251</v>
+        <v>232</v>
       </c>
       <c r="F31" s="21">
-        <v>411</v>
+        <v>471</v>
       </c>
       <c r="G31" s="22" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H31" s="16">
         <v>0</v>
@@ -2210,25 +2219,25 @@
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B32" s="16">
         <v>100</v>
       </c>
       <c r="C32" s="19">
-        <v>122</v>
+        <v>114</v>
       </c>
       <c r="D32" s="16">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="E32" s="20">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="F32" s="21">
-        <v>564</v>
+        <v>437</v>
       </c>
       <c r="G32" s="22" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H32" s="16">
         <v>0</v>
@@ -2239,25 +2248,25 @@
     </row>
     <row r="33" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B33" s="16">
         <v>100</v>
       </c>
       <c r="C33" s="19">
-        <v>134</v>
+        <v>113</v>
       </c>
       <c r="D33" s="16">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="E33" s="20">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="F33" s="21">
-        <v>647</v>
+        <v>502</v>
       </c>
       <c r="G33" s="22" t="s">
-        <v>122</v>
+        <v>95</v>
       </c>
       <c r="H33" s="16">
         <v>0</v>
@@ -2274,16 +2283,16 @@
         <v>100</v>
       </c>
       <c r="C34" s="19">
-        <v>133</v>
+        <v>121</v>
       </c>
       <c r="D34" s="16">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="E34" s="20">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="F34" s="21">
-        <v>538</v>
+        <v>445</v>
       </c>
       <c r="G34" s="22" t="s">
         <v>124</v>
@@ -2303,19 +2312,19 @@
         <v>100</v>
       </c>
       <c r="C35" s="19">
-        <v>120</v>
+        <v>130</v>
       </c>
       <c r="D35" s="16">
         <v>58</v>
       </c>
       <c r="E35" s="20">
-        <v>269</v>
+        <v>248</v>
       </c>
       <c r="F35" s="21">
-        <v>541</v>
+        <v>484</v>
       </c>
       <c r="G35" s="22" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H35" s="16">
         <v>0</v>
@@ -2326,25 +2335,25 @@
     </row>
     <row r="36" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B36" s="16">
         <v>100</v>
       </c>
       <c r="C36" s="19">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="D36" s="16">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="E36" s="20">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="F36" s="21">
-        <v>457</v>
+        <v>418</v>
       </c>
       <c r="G36" s="22" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H36" s="16">
         <v>0</v>
@@ -2355,25 +2364,25 @@
     </row>
     <row r="37" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B37" s="16">
         <v>100</v>
       </c>
       <c r="C37" s="19">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D37" s="16">
-        <v>51</v>
+        <v>57</v>
       </c>
       <c r="E37" s="20">
-        <v>237</v>
+        <v>267</v>
       </c>
       <c r="F37" s="21">
-        <v>447</v>
+        <v>638</v>
       </c>
       <c r="G37" s="22" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H37" s="16">
         <v>0</v>
@@ -2384,25 +2393,25 @@
     </row>
     <row r="38" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B38" s="16">
         <v>100</v>
       </c>
       <c r="C38" s="19">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="D38" s="16">
-        <v>56</v>
+        <v>47</v>
       </c>
       <c r="E38" s="20">
-        <v>230</v>
+        <v>259</v>
       </c>
       <c r="F38" s="23">
         <v>1500</v>
       </c>
       <c r="G38" s="22" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H38" s="16">
         <v>1</v>
@@ -2413,25 +2422,25 @@
     </row>
     <row r="39" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B39" s="16">
         <v>100</v>
       </c>
       <c r="C39" s="19">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D39" s="16">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="E39" s="20">
-        <v>234</v>
+        <v>259</v>
       </c>
       <c r="F39" s="21">
-        <v>494</v>
+        <v>511</v>
       </c>
       <c r="G39" s="22" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H39" s="16">
         <v>0</v>
@@ -2442,25 +2451,25 @@
     </row>
     <row r="40" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B40" s="16">
         <v>100</v>
       </c>
       <c r="C40" s="19">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D40" s="16">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E40" s="20">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="F40" s="21">
-        <v>462</v>
+        <v>619</v>
       </c>
       <c r="G40" s="22" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H40" s="16">
         <v>0</v>
@@ -2471,25 +2480,25 @@
     </row>
     <row r="41" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B41" s="16">
         <v>100</v>
       </c>
       <c r="C41" s="19">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="D41" s="16">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E41" s="20">
-        <v>269</v>
+        <v>255</v>
       </c>
       <c r="F41" s="21">
-        <v>541</v>
+        <v>572</v>
       </c>
       <c r="G41" s="22" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H41" s="16">
         <v>0</v>
@@ -2500,25 +2509,25 @@
     </row>
     <row r="42" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B42" s="16">
         <v>100</v>
       </c>
       <c r="C42" s="19">
-        <v>123</v>
+        <v>133</v>
       </c>
       <c r="D42" s="16">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E42" s="20">
-        <v>257</v>
+        <v>243</v>
       </c>
       <c r="F42" s="21">
-        <v>580</v>
+        <v>444</v>
       </c>
       <c r="G42" s="22" t="s">
-        <v>139</v>
+        <v>91</v>
       </c>
       <c r="H42" s="16">
         <v>0</v>
@@ -2535,16 +2544,16 @@
         <v>100</v>
       </c>
       <c r="C43" s="19">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="D43" s="16">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="E43" s="20">
-        <v>234</v>
+        <v>244</v>
       </c>
       <c r="F43" s="21">
-        <v>414</v>
+        <v>590</v>
       </c>
       <c r="G43" s="22" t="s">
         <v>141</v>
@@ -2564,19 +2573,19 @@
         <v>100</v>
       </c>
       <c r="C44" s="19">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="D44" s="16">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E44" s="20">
-        <v>250</v>
+        <v>243</v>
       </c>
       <c r="F44" s="21">
-        <v>602</v>
+        <v>557</v>
       </c>
       <c r="G44" s="22" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H44" s="16">
         <v>0</v>
@@ -2587,25 +2596,25 @@
     </row>
     <row r="45" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="B45" s="16">
         <v>100</v>
       </c>
       <c r="C45" s="19">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="D45" s="16">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="E45" s="20">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="F45" s="21">
-        <v>573</v>
+        <v>425</v>
       </c>
       <c r="G45" s="22" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H45" s="16">
         <v>0</v>
@@ -2616,25 +2625,25 @@
     </row>
     <row r="46" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A46" s="16" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B46" s="16">
         <v>100</v>
       </c>
       <c r="C46" s="19">
-        <v>130</v>
+        <v>110</v>
       </c>
       <c r="D46" s="16">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="E46" s="20">
-        <v>242</v>
+        <v>250</v>
       </c>
       <c r="F46" s="21">
-        <v>523</v>
+        <v>512</v>
       </c>
       <c r="G46" s="22" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H46" s="16">
         <v>0</v>
@@ -2645,25 +2654,25 @@
     </row>
     <row r="47" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A47" s="16" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B47" s="16">
         <v>100</v>
       </c>
       <c r="C47" s="19">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D47" s="16">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E47" s="20">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="F47" s="21">
-        <v>632</v>
+        <v>530</v>
       </c>
       <c r="G47" s="22" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H47" s="16">
         <v>0</v>
@@ -2674,25 +2683,25 @@
     </row>
     <row r="48" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A48" s="16" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B48" s="16">
         <v>100</v>
       </c>
       <c r="C48" s="19">
-        <v>130</v>
+        <v>119</v>
       </c>
       <c r="D48" s="16">
         <v>56</v>
       </c>
       <c r="E48" s="20">
-        <v>234</v>
+        <v>266</v>
       </c>
       <c r="F48" s="21">
-        <v>405</v>
+        <v>462</v>
       </c>
       <c r="G48" s="22" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H48" s="16">
         <v>0</v>
@@ -2703,25 +2712,25 @@
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" s="16" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B49" s="16">
         <v>100</v>
       </c>
       <c r="C49" s="19">
-        <v>127</v>
+        <v>115</v>
       </c>
       <c r="D49" s="16">
-        <v>53</v>
+        <v>46</v>
       </c>
       <c r="E49" s="20">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="F49" s="21">
-        <v>535</v>
+        <v>565</v>
       </c>
       <c r="G49" s="22" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H49" s="16">
         <v>0</v>
@@ -2732,25 +2741,25 @@
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A50" s="16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B50" s="16">
         <v>100</v>
       </c>
       <c r="C50" s="19">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="D50" s="16">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="E50" s="20">
         <v>253</v>
       </c>
       <c r="F50" s="21">
-        <v>503</v>
+        <v>436</v>
       </c>
       <c r="G50" s="22" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H50" s="16">
         <v>0</v>
@@ -2761,25 +2770,25 @@
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A51" s="16" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B51" s="16">
         <v>100</v>
       </c>
       <c r="C51" s="19">
-        <v>127</v>
+        <v>118</v>
       </c>
       <c r="D51" s="16">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="E51" s="20">
-        <v>243</v>
+        <v>256</v>
       </c>
       <c r="F51" s="21">
-        <v>568</v>
+        <v>466</v>
       </c>
       <c r="G51" s="22" t="s">
-        <v>156</v>
+        <v>68</v>
       </c>
       <c r="H51" s="16">
         <v>0</v>
@@ -2796,19 +2805,19 @@
         <v>100</v>
       </c>
       <c r="C52" s="19">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="D52" s="16">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="E52" s="20">
-        <v>242</v>
+        <v>256</v>
       </c>
       <c r="F52" s="21">
-        <v>436</v>
+        <v>532</v>
       </c>
       <c r="G52" s="22" t="s">
-        <v>127</v>
+        <v>158</v>
       </c>
       <c r="H52" s="16">
         <v>0</v>
@@ -2819,7 +2828,7 @@
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A53" s="16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B53" s="16">
         <v>100</v>
@@ -2828,16 +2837,16 @@
         <v>129</v>
       </c>
       <c r="D53" s="16">
-        <v>58</v>
+        <v>49</v>
       </c>
       <c r="E53" s="20">
-        <v>245</v>
+        <v>269</v>
       </c>
       <c r="F53" s="21">
-        <v>602</v>
+        <v>496</v>
       </c>
       <c r="G53" s="22" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H53" s="16">
         <v>0</v>
@@ -2848,25 +2857,25 @@
     </row>
     <row r="54" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A54" s="16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B54" s="16">
         <v>100</v>
       </c>
       <c r="C54" s="19">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="D54" s="16">
-        <v>58</v>
+        <v>45</v>
       </c>
       <c r="E54" s="20">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="F54" s="21">
-        <v>576</v>
+        <v>403</v>
       </c>
       <c r="G54" s="22" t="s">
-        <v>118</v>
+        <v>162</v>
       </c>
       <c r="H54" s="16">
         <v>0</v>
@@ -2877,25 +2886,25 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="B55" s="16">
         <v>100</v>
       </c>
       <c r="C55" s="19">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="D55" s="16">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="E55" s="20">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="F55" s="21">
-        <v>442</v>
+        <v>439</v>
       </c>
       <c r="G55" s="22" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="H55" s="16">
         <v>0</v>
@@ -2906,25 +2915,25 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" s="16" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="B56" s="16">
         <v>100</v>
       </c>
       <c r="C56" s="19">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="D56" s="16">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="E56" s="20">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="F56" s="21">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="G56" s="22" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H56" s="16">
         <v>0</v>
@@ -2935,25 +2944,25 @@
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A57" s="16" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="B57" s="16">
         <v>100</v>
       </c>
       <c r="C57" s="19">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="D57" s="16">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E57" s="20">
-        <v>253</v>
+        <v>240</v>
       </c>
       <c r="F57" s="21">
-        <v>624</v>
+        <v>606</v>
       </c>
       <c r="G57" s="22" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H57" s="16">
         <v>0</v>
@@ -2964,25 +2973,25 @@
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A58" s="16" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="B58" s="16">
         <v>100</v>
       </c>
       <c r="C58" s="19">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D58" s="16">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E58" s="20">
-        <v>268</v>
+        <v>246</v>
       </c>
       <c r="F58" s="21">
-        <v>559</v>
+        <v>483</v>
       </c>
       <c r="G58" s="22" t="s">
-        <v>144</v>
+        <v>89</v>
       </c>
       <c r="H58" s="16">
         <v>0</v>
@@ -2993,25 +3002,25 @@
     </row>
     <row r="59" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A59" s="16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="B59" s="16">
         <v>100</v>
       </c>
       <c r="C59" s="19">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D59" s="16">
-        <v>48</v>
+        <v>57</v>
       </c>
       <c r="E59" s="20">
-        <v>263</v>
+        <v>251</v>
       </c>
       <c r="F59" s="21">
-        <v>407</v>
+        <v>626</v>
       </c>
       <c r="G59" s="22" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="H59" s="16">
         <v>0</v>
@@ -3022,25 +3031,25 @@
     </row>
     <row r="60" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A60" s="16" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="B60" s="16">
         <v>100</v>
       </c>
       <c r="C60" s="19">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="D60" s="16">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="E60" s="20">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="F60" s="21">
-        <v>451</v>
+        <v>605</v>
       </c>
       <c r="G60" s="22" t="s">
-        <v>120</v>
+        <v>173</v>
       </c>
       <c r="H60" s="16">
         <v>0</v>
@@ -3051,25 +3060,25 @@
     </row>
     <row r="61" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A61" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B61" s="16">
         <v>100</v>
       </c>
       <c r="C61" s="19">
-        <v>126</v>
+        <v>114</v>
       </c>
       <c r="D61" s="16">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E61" s="20">
-        <v>264</v>
+        <v>237</v>
       </c>
       <c r="F61" s="21">
-        <v>558</v>
+        <v>626</v>
       </c>
       <c r="G61" s="22" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="H61" s="16">
         <v>0</v>

</xml_diff>